<commit_message>
Run accounting analyzer on organized files
</commit_message>
<xml_diff>
--- a/08_Reports - Доклади - Berichte/Accounting_Cash_Flow/employee_timeline.xlsx
+++ b/08_Reports - Доклади - Berichte/Accounting_Cash_Flow/employee_timeline.xlsx
@@ -55,7 +55,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/10001_09-2024_Brutto_NettoProbe_00051_QZ1.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/02_Payroll/10001_09-2024_Brutto_NettoProbe_00051_QZ1.pdf</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -82,7 +82,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/10001_09-2024_Brutto_NettoProbe_00107_QZ1.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/02_Payroll/10001_09-2024_Brutto_NettoProbe_00107_QZ1.pdf</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -94,7 +94,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2025-01</t>
+          <t>2021-02</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -104,12 +104,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Euro, Tsd; Kilometer, St; Tage, Km; Tausend Euro, Mio</t>
+          <t>ADAC, Hansastr; MP, MARTIN ZAHARIEVSOZIALVERSICHER; Rundfunk ARD, ZDF; ZAHARIEV, MARTIN ADAC VERSICHER</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/12-2024_Brutto_Netto_00090_X0B.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/02-2021 #9109.pdf</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -121,22 +121,22 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2024-02</t>
+          <t>2022-03</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>10</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Avis Budget Autovermietung Verwaltungsgesellschaft mbH, Oberursel; KG, Amtsgericht Bad Homburg v; OBERURSEL, GERMANY; Sollten Sie Fragen, Wünsche oder auch Beanstandungen haben; Wir hoffen, Sie bald wieder bei uns begrüssen zu dürfen; ZAHARIEV,MARTIN; ZAHARIEV,MARTIN Gefahrene Entfernung</t>
+          <t>ADAC, Hansastr; ALEX Chemnitz, Galerie Roter Turm; ARD, ZDF; Burger King, FOOD STAR GmbH; GLOBUS SBW, CHEMNITZ; Globus SBW, Chemnitz; Gutschrift Darling züruck , Danke Mersi; MP, INH; MP, MARTIN ZAHARIEVSOZIALVERSICHER; ZAHARIEV, MARTIN ADAC VERSICHER</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/307538032.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/02-2022 #9109.pdf</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -148,76 +148,76 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t/>
+          <t>2023-03</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t/>
+          <t>9</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t/>
+          <t>ADAC Versicherung AG, Hansastr; ADAC, Hansastr; ALEX Chemnitz, Galerie Roter Turm; ARD, ZDF; Burger King, FOOD STAR GmbH; EUR, SOL; KG, Ihr Einkauf bei Parf; MP, INH; ZAHARIEV, MARTIN ADAC VERSICHER</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/38389 - Vorgangsmappe Lohn - Aktualisiert- Auszahlungen Inflationsprämie.xlsx</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/02-2023 #9109.pdf</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2025-05</t>
+          <t>2021-04</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t/>
+          <t>4</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t/>
+          <t>ADAC, Hansastr; MP, MARTIN ZAHARIEVSOZIALVERSICHER; Rundfunk ARD, ZDF; ZAHARIEV, MARTIN ADAC VERSICHER</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/38389 - Vorgangsmappe Lohn - Contributions 28.05.2025.docx</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/04-2021 #9109.pdf</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2024-06</t>
+          <t>2022-05</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Brunettin, Mari; Marco Brunettin; Marco Brunettin, LL</t>
+          <t>ADAC, Hansastr; ALEX Chemnitz, Galerie Roter Turm; ARD, ZDF; BUONO, CHEMNITZ; GLOBUS SBW, CHEMNITZ; Gutschrift Darling züruck , Danke Mersi; MP, INH; Reece Upadhyay, Ihr Einkauf bei R; ZAHARIEV, MARTIN ADAC VERSICHER</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/42585 - Rechnung 240587_2024 vom 29.06.2024, Aufträge 31_24, 33_23, 33_24, 34_24, Mandant 42303-1.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/04-2022 #9109.pdf</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -229,22 +229,22 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2025-08</t>
+          <t>2021-06</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Auftrag unseres Mandanten, Martin Zahariev; Brunettin, Marilie</t>
+          <t>ADAC, Hansastr; ARD, ZDF; DANKE, IHR LIDL; MP, MARTIN ZAHARIEVSOZIALVERSICHER; Simply NetTrade GmbH, Ihr Einkauf bei Simply NetTrade Gmb; ZAHARIEV, MARTIN ADAC VERSICHER</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/89878877, Antrag auf Ratenzahlung.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/06-2021 #9109.pdf</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -256,22 +256,22 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2004-12</t>
+          <t>2022-07</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Brunettin, Marco; Kind regards, Marco; Marco Brunettin, LL</t>
+          <t>ADAC, Hansastr; ALEX Chemnitz, Galerie Roter Turm; ARD, ZDF; AUTO CENTER SUED, CHEMNITZ; BRAZIL OHG, CHEMNITZ; BUONO, CHEMNITZ; MP, INH; Reece Upadhyay, Ihr Einkauf bei R; ZAHARIEV, MARTIN ADAC VERSICHER</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/Accountings 01-2025.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/06-2022 #9109.pdf</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -283,22 +283,22 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2004-12</t>
+          <t>2021-07</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Brunettin, Marco; Kind regards, Marco; Marco Brunettin, LL</t>
+          <t>ADAC, Hansastr; ARD, ZDF; Burger King, FOOD STAR GmbH; DANKE, IHR LIDL; MP, MARTIN ZAHARIEVSOZIALVERSICHER; Simply NetTrade GmbH, Ihr Einkauf bei Simply NetTrade Gmb; ZAHARIEV, MARTIN ADAC VERSICHER</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/Accountings 02-2024.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/07-2021 #9109.pdf</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -310,22 +310,22 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2004-12</t>
+          <t>2022-08</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Brunettin, Marco; Kind regards, Marco; Marco Brunettin, LL</t>
+          <t>ADAC, Hansastr; ALEX Chemnitz, Galerie Roter Turm; ARD, ZDF; AUTO CENTER SUED, CHEMNITZ; MP, INH; ZAHARIEV, MARTIN ADAC VERSICHER</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/Accountings 02-2025.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/07-2022 #9109.pdf</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -337,22 +337,22 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2004-12</t>
+          <t>2021-08</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Brunettin, Marco; Kind regards, Marco; Marco Brunettin, LL</t>
+          <t>ADAC, Hansastr; ARD, ZDF; BRAZIL OHG, CHEMNITZ; Burger King, FOOD STAR GmbH; DANKE, IHR LIDL; MP, MARTIN ZAHARIEVSOZIALVERSICHER; ZAHARIEV, MARTIN ADAC VERSICHER</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/Accountings 03-2024.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/09-2021 #9109.pdf</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -364,22 +364,22 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2024-09</t>
+          <t>2022-10</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Brunettin, Marco; Kind regards, Marco; Marco Brunettin, LL</t>
+          <t>ADAC, Hansastr; AGIP,ANSBACHER STR; AGIP,NUERNBERG; ALEX Chemnitz, Galerie Roter Turm; ARD, ZDF; AUTO CENTER SUED, CHEMNITZ; BUONO, CHEMNITZ; Burger King, FOOD STAR GmbH; MP, INH; ZAHARIEV, MARTIN ADAC VERSICHER</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/Accountings 04-2024.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/10-2022 #9109.pdf</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -391,22 +391,22 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2004-12</t>
+          <t>2021-08</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Brunettin, Marco; Kind regards, Marco; Marco Brunettin, LL</t>
+          <t>ADAC, Hansastr; ARD, ZDF; FAVORIT MP, MARTINSOZIALVERSICHERU; MP, MARTIN ZAHARIEVSOZIALVERSICHER; MP, MARTIN ZAHARIEVSOZIALVERSICHERU; ZAHARIEV, MARTIN ADAC VERSICHER; Überweisung Kirev,Kosta</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/Accountings 05-2024.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/11-2021 #9109.pdf</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -418,22 +418,22 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2004-12</t>
+          <t>2021-12</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>11</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Brunettin, Marco; Marco Brunettin, LL</t>
+          <t>ADAC, Hansastr; ARD, ZDF; Burger King, FOOD STAR GmbH; EUR, UMS; FAVORIT MP, MARTINSOZIALVERSICHERU; GLOBUS SBW, CHEMNITZ; Globus SBW, Chemnitz; MP, MARTIN ZAHARIEVSOZIALVERSICHER; MP, MARTIN ZAHARIEVSOZIALVERSICHERU; ZAHARIEV, MARTIN ADAC VERSICHER; Überweisung Kirev,Kosta</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/Accountings 06-2024.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/12-2021 #9109.pdf</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -445,22 +445,22 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2004-12</t>
+          <t>2022-12</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>11</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Brunettin, Marco; Kind regards, Marco; Marco Brunettin, LL</t>
+          <t>ADAC, Hansastr; AGIP,ANSBACHER STR; AGIP,NUERNBERG; ALEX Chemnitz, Galerie Roter Turm; ARD, ZDF; AUTO CENTER SUED, CHEMNITZ; BUONO, CHEMNITZ; Burger King, FOOD STAR GmbH; KG, Ihr Einkauf bei Parf; MP, INH; ZAHARIEV, MARTIN ADAC VERSICHER</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/Accountings 07-2024.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/12-2022 #9109.pdf</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -472,22 +472,22 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2024-11</t>
+          <t>2025-01</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Brunettin, Marco; Kind regards, Marco; Marco Brunettin, LL</t>
+          <t>Euro, Tsd; Kilometer, St; Tage, Km; Tausend Euro, Mio</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/Accountings 09-2024.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/12-2024_Brutto_Netto_00090_X0B.pdf</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -499,49 +499,49 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2004-12</t>
+          <t>2025-05</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2</t>
+          <t/>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Brunettin, Marco; Marco Brunettin, LL</t>
+          <t/>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/Accountings 10-2024.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/38389 - Vorgangsmappe Lohn - Contributions 28.05.2025.docx</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>LOW</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2025-12</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Brunettin, Marco; Kind regards, Marco; Marco Brunettin, LL</t>
+          <t>Betreuung durch den ASD, Bescheid; EUR Warenlieferung, Forderung aus; Feuerwehr Zwickau, Kennzeichen; Ieva Meilutyte, Stefan Mihaila; Säumniszuschläge, Kosten; Säumniszuschläge, Nachzahlungszinsen und; Säumniszuschläge, Zinsen; Ventsislav Kostov, Ionel Neamtu; ZV-Sache, AG Chemnitz; Zahariev, Martin</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/Accountings 11-2024.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/Tabelle nach § 175 InsO mit Grund des Bestreitens.pdf</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -558,17 +558,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Brunettin, Marco; Kind regards, Marco; Marco Brunettin, LL</t>
+          <t>Euro, Tsd; Kilometer, St; Tage, Km; Tausend Euro, Mio</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/Accountings 12-2024.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/04_Health_Insurance/Vasilev_Test Pay Slip.pdf</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -580,103 +580,103 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2025-11</t>
+          <t/>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>3</t>
+          <t/>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Brunettin, Marco; Brunettin, Marilie; Hello again, I called the AOK Plus</t>
+          <t/>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/Aok plus.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/05_Taxes/38389 - Vorgangsmappe Lohn - 38389 - Aktualisiert- Auszahlungen Inflationsprämie.xlsx</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>LOW</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2024-09</t>
+          <t>2023-10</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t/>
+          <t>2</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t/>
+          <t>Marco Brunettin; Marco Brunettin, LL</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/CarlundCarla_RG424005125.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/05_Taxes/90f3df27-1ca1-4b3a-9f1b-e33ffd37f10a.pdf</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2024-09</t>
+          <t/>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t/>
+          <t>14</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t/>
+          <t>Boulevard Royal, L; Der Verkäufer behält sich vor, Verarbeitungsaufträge abzulehnen; E-Mail, Fax oder Brief; EE Amsterdam, Niederlande; Grafiken in den vom Verkäufer vorgegebenen Dateiformaten, Formatierungen; Kennedy, L; Reklamationen, Widerrufserklärungen und; Reklamationen, Widerrufserklärungen und -zusendungen oder Gutschriften; Stockholm, Schweden; Urheber-, Marken- und Persönlichkeitsrechte; Versendung, Retouren; Ware, Lieferzeit; Zahlungsabwicklung über die TeamBank AG Nürnberg, Beuthener Straße; Überweisungsgebühren, Wechselkursgebühren</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/CarlundCarla_RG424005157.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/05_Taxes/agb_doc.pdf</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2004-12</t>
+          <t>2025-09</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Brunettin, Marilie; Hello again, I have spoken to the DAK</t>
+          <t>Autoverwertung-Oskar, Schulstr</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/DAK.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/05_Taxes/Rechnung_RE058675_11.08.2025.pdf</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -688,22 +688,22 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2024-07</t>
+          <t/>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Logistikbetrieb Weißlog, Hohensteiner Str</t>
+          <t>Herleshausen, Deutschland; Post versandter Brief, Telefax oder E-Mail; Weber GmbH, Sülzbach</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/Docutain Dokument.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/05_Taxes/widerruf_doc.pdf</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -715,22 +715,22 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2024-10</t>
+          <t>2022-11</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Goetz, Schneeberg; Logistikbetrieb Weißflog, Hohensteiner Str; Steuerbereinigter Schadenersatz, Schadenbetrag ohne Mehrwertsteuer</t>
+          <t>Parfumerie Douglas GmbH, Ihr Eink auf bei Parfumeri; Parfumerie Douglas GmbH, Ihr Einkau; Skull Sh aver EU Ltd, Ihr Ei; Skull Shaver EU Ltd, Ihr Einkauf bei Skull Shaver EU Lt</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/Gutschrift 34-2024 Zahariev Martin 04.10.2024.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/01-2023 #9120.pdf</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -742,22 +742,22 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2025-06</t>
+          <t>2022-02</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Steuerbereinigter Schadenersatz, Schadenbetrag ohne Mehrwertsteuer</t>
+          <t>ALEX Chemnitz, Galerie Roter Turm; Burger King, FOOD STAR GmbH; Limited, Ih</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/gutschrift 71 2025 zahariev Sendungsverlust.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/02-2022 #9120.pdf</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -769,22 +769,22 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2025-11</t>
+          <t>2022-04</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Brunettin, Marilie</t>
+          <t>ALEX Chemnitz, Galerie Roter Turm; AUTODOC AG, Ihr Einkau; Burger King, FOOD STAR GmbH; Dott, Ihr Einkauf bei Dott; EUR, Tra; Limited, Ih; Tier Mobility GmbH, Ihr Einkauf b</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/Health insurance fund reimbursements.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/04-2022 #9120.pdf</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -796,22 +796,22 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2024-09</t>
+          <t>2022-06</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Brunettin, Marilie</t>
+          <t>ALEX Chemnitz, Galerie Roter Turm; AUTO CENTER SUED, CHEMNITZ; AUTODOC AG, Ihr Einkau; Dott, Ihr Einkauf bei Dott; Tier Mobility GmbH, Ihr Einkauf b</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/Ihre Lohnauswertungen.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/06-2022 #9120.pdf</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -823,22 +823,22 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2025-08</t>
+          <t>2022-08</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Timothy Grygotis, Julia von SpechtSitz</t>
+          <t>ADAC, Hansastr; ALEX Chemnitz, Galerie Roter Turm</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/KD-Nr. 550980 - Pre-Not._Nr. 6102600491.PDF</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/07-2022 #9120.pdf</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -850,22 +850,22 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2025-09</t>
+          <t>2022-10</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Timothy Grygotis, Julia von SpechtSitz</t>
+          <t>ADAC, Hansastr; AG, Ihr Einkauf bei AUTODOC AG; ALEX Chemnitz, Galerie Roter Turm</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/KD-Nr. 550980 - Pre-Not._Nr. 6102659867.PDF</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/10-2022 #9120.pdf</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -877,22 +877,22 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2025-09</t>
+          <t>2022-12</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Timothy Grygotis, Julia von SpechtSitz</t>
+          <t>AG, Ihr Einkauf bei AUTODOC AG; EU Ltd, Ihr Einkauf bei Skull; GmbH, Ihr Einkauf bei Parfumerie Do; Parfumerie Douglas GmbH, Ihr Eink</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/KD-Nr. 550980 - Pre-Not._Nr. 6102665850.PDF</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/12-2022 #9120.pdf</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -904,22 +904,22 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2025-09</t>
+          <t>2024-01</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Timothy Grygotis, Julia von SpechtSitz</t>
+          <t>Akkreditiert durch DAkkS, Registriernummer; Berlin-Charlottenburg, HRB; Präqualifikation Kurier-, Express- und Paketdienstleistern i; ZERTIFIZIERUNG BAU GMBH, Kronenstraße</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/KD-Nr. 550980 - Pre-Not._Nr. 6102698674.PDF</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/20240123_60222_10160_Rechnung.pdf</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -931,22 +931,22 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2025-09</t>
+          <t>2025-08</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Brunettin, Marilie; Good morning Martin, I have just called the KKH</t>
+          <t>Timothy Grygotis, Julia von SpechtSitz</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/KKH1.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/KD-Nr. 550980 - Pre-Not._Nr. 6102600491.PDF</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -958,7 +958,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2025-11</t>
+          <t>2025-09</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -968,12 +968,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Brunettin, Marilie</t>
+          <t>Timothy Grygotis, Julia von SpechtSitz</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/Mahnbescheid Amtsgericht Euskirchen _ AXA.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/KD-Nr. 550980 - Pre-Not._Nr. 6102659867.PDF</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -985,22 +985,22 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2025-02</t>
+          <t>2025-09</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Logistikbetrieb Weißflog, Hohensteiner Str; Steuerbereinigter Schadenersatz, Schadenbetrag ohne Mehrwertsteuer</t>
+          <t>Timothy Grygotis, Julia von SpechtSitz</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/Martin Zahariev Gutschrift 51 17.02.2025.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/KD-Nr. 550980 - Pre-Not._Nr. 6102665850.PDF</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1012,22 +1012,22 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2025-03</t>
+          <t>2025-09</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Logistikbetrieb Weißflog, Hohensteiner Str; Steuerbereinigter Schadenersatz, Schadenbetrag ohne Mehrwertsteuer</t>
+          <t>Timothy Grygotis, Julia von SpechtSitz</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/Martin Zahariev Gutschrift 55 08.03.2025.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/KD-Nr. 550980 - Pre-Not._Nr. 6102698674.PDF</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1039,7 +1039,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2058-08</t>
+          <t/>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1049,12 +1049,12 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Logistikbetrieb Weißflog, Hohensteiner Str</t>
+          <t>Andreas Weber, Horst WeberHandelsregister</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/Martin Zahariev Transporte 2058 08.03.2025 Scannermiete.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/Rechnung RE211073-1.pdf</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -1066,22 +1066,22 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2025-10</t>
+          <t/>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Brunettin, Marilie; Good morning Martin, I have just called the KKH; When it is paid, I can ask for the Unbedenklichkeitsbescheingungen</t>
+          <t>Andreas Weber, Horst WeberHandelsregister</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/original_msg(2).eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/Rechnung RE211073.pdf</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1093,7 +1093,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2024-07</t>
+          <t>2025-09</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1103,12 +1103,12 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Brunettin, Marilie</t>
+          <t>Timothy Grygotis, Julia von Specht</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/Petya Stefanova AOK.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/Rücklastschrift _ Ihre KD-Nr. 550980-1.PDF</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1120,22 +1120,22 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2024-08</t>
+          <t>2025-09</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Chemnitz , Sachs; Motoren-Frech, Uwe; Thomas Frech GbR, Hohensteiner Straße</t>
+          <t>Timothy Grygotis, Julia von Specht</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/RE-53380_2024 13.08.2024 09_17_16.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/Rücklastschrift _ Ihre KD-Nr. 550980-2.PDF</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -1147,22 +1147,22 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2024-09</t>
+          <t>2025-09</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Chemnitz , Sachs; Motoren-Frech, Uwe; Thomas Frech GbR, Hohensteiner Straße</t>
+          <t>Timothy Grygotis, Julia von Specht</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/RE-53652_2024 20.09.2024 10_56_50.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/Rücklastschrift _ Ihre KD-Nr. 550980.PDF</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -1174,22 +1174,22 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t/>
+          <t>2024-02</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Andreas Weber, Horst WeberHandelsregister</t>
+          <t>Avis Budget Autovermietung Verwaltungsgesellschaft mbH, Oberursel; KG, Amtsgericht Bad Homburg v; OBERURSEL, GERMANY; Sollten Sie Fragen, Wünsche oder auch Beanstandungen haben; Wir hoffen, Sie bald wieder bei uns begrüssen zu dürfen; ZAHARIEV,MARTIN; ZAHARIEV,MARTIN Gefahrene Entfernung</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/Rechnung RE211073-1.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/307538032.pdf</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -1201,22 +1201,22 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t/>
+          <t>2023-12</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Andreas Weber, Horst WeberHandelsregister</t>
+          <t>Marco Brunettin; Marco Brunettin, LL</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/Rechnung RE211073.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/39739 - Rechnung 231128_2023 vom 28.12.2023, Aufträge 31_23, 32_23, 33_23, 34_23, 50_23, 98_23, Mandant 42303.pdf</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -1228,22 +1228,22 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2025-09</t>
+          <t>2024-02</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Autoverwertung-Oskar, Schulstr</t>
+          <t>Marco Brunettin; Marco Brunettin, LL</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/Rechnung_RE058675_11.08.2025.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/40579 - Rechnung 240155_2024 vom 17.02.2024, Aufträge 31_23, 33_23, 34_23, Mandant 42303.pdf</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -1255,22 +1255,22 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2025-09</t>
+          <t>2024-01</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Timothy Grygotis, Julia von Specht</t>
+          <t>Brunettin, Mari; Marco Brunettin; Marco Brunettin, LL</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/Rücklastschrift _ Ihre KD-Nr. 550980-1.PDF</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/40850 - Rechnung 240213_2024 vom 29.01.2024, Aufträge 31_24, 32_23, 33_23, 33_24, 34_24, 98_24, Mandant 42303.pdf</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -1282,22 +1282,22 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2025-09</t>
+          <t>2024-03</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Timothy Grygotis, Julia von Specht</t>
+          <t>Brunettin, Mari; Marco Brunettin; Marco Brunettin, LL</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/Rücklastschrift _ Ihre KD-Nr. 550980-2.PDF</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/41261 - Rechnung 240303_2024 vom 27.03.2024, Aufträge 31_24, 33_24, 34_24, Mandant 42303.pdf</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -1309,22 +1309,22 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2025-09</t>
+          <t>2024-04</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Timothy Grygotis, Julia von Specht</t>
+          <t>Brunettin, Mari; Marco Brunettin; Marco Brunettin, LL</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/Rücklastschrift _ Ihre KD-Nr. 550980.PDF</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/41683 - Rechnung 240393_2024 vom 30.04.2024, Aufträge 31_24, 32_24, 33_24, 34_24, 98_24, Mandant 42303.pdf</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -1336,22 +1336,22 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2024-05</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Betreuung durch den ASD, Bescheid; EUR Warenlieferung, Forderung aus; Feuerwehr Zwickau, Kennzeichen; Ieva Meilutyte, Stefan Mihaila; Säumniszuschläge, Kosten; Säumniszuschläge, Nachzahlungszinsen und; Säumniszuschläge, Zinsen; Ventsislav Kostov, Ionel Neamtu; ZV-Sache, AG Chemnitz; Zahariev, Martin</t>
+          <t>Brunettin, Mari; Marco Brunettin; Marco Brunettin, LL</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/Tabelle nach § 175 InsO mit Grund des Bestreitens.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/42108 - Rechnung 240498_2024 vom 30.05.2024, Aufträge 21_24, 31_24, 32_24, 33_24, 34_24, Mandant 42303.pdf</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -1363,22 +1363,22 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2023-10</t>
+          <t>2024-06</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Dennis Kollmann, Marco Schlüter</t>
+          <t>Brunettin, Mari; Marco Brunettin; Marco Brunettin, LL</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/Unternehmerabrechnung - VP 120-2300157425.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/42585 - Rechnung 240587_2024 vom 29.06.2024, Aufträge 31_24, 33_23, 33_24, 34_24, Mandant 42303-1.pdf</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -1390,22 +1390,22 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2023-10</t>
+          <t>2024-07</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Dennis Kollmann, Marco Schlüter</t>
+          <t>Brunettin, Mari; EURPQ, Matodiev wage statement; Marco Brunettin; Marco Brunettin, LL; Stefanova, Yordanov</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/Unternehmerabrechnung - VP 120-2300157934.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/43029 - Rechnung 240697_2024 vom 31.07.2024, Aufträge 21_23, 21_24, 31_22, 31_23, 31_24, 33_24, 34_24, Mandant 42303.pdf</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -1417,22 +1417,22 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2024-01</t>
+          <t>2024-08</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Dennis Kollmann, Marco Schlüter</t>
+          <t>Brunettin, Mari; Marco Brunettin; Marco Brunettin, LL</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/Unternehmerabrechnung - VP 120-2400001108-1.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/43617 - Rechnung 240857_2024 vom 30.08.2024, Aufträge 31_24, 32_24, 33_24, 34_24, Mandant 42303.pdf</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -1444,22 +1444,22 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2024-02</t>
+          <t>2024-10</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Dennis Kollmann, Marco Schlüter</t>
+          <t>Brunettin, Mari; Marco Brunettin; Marco Brunettin, LL</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/Unternehmerabrechnung - VP 120-2400017841.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/44458 - Rechnung 241068_2024 vom 30.10.2024, Aufträge 31_24, 33_24, 34_24, Mandant 42303.pdf</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -1471,22 +1471,22 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2024-02</t>
+          <t>2024-11</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Dennis Kollmann, Marco Schlüter</t>
+          <t>Brunettin, Mari; Marco Brunettin; Marco Brunettin, LL</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/Unternehmerabrechnung - VP 120-2400018211.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/45027 - Rechnung 241185_2024 vom 29.11.2024, Aufträge 31_24, 33_24, 34_24, Mandant 42303.pdf</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -1498,22 +1498,22 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2025-12</t>
+          <t>2024-12</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Euro, Tsd; Kilometer, St; Tage, Km; Tausend Euro, Mio</t>
+          <t>Brunettin, Mari; Marco Brunettin; Marco Brunettin, LL</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/Vasilev_Test Pay Slip.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/45474 - Rechnung 241289_2024 vom 27.12.2024, Aufträge 21_24, 31_24, 32_24, 33_24, 34_24, 35_21, 35_24, 50_24, 98_24, Mandant 42303.pdf</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -1525,22 +1525,22 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2025-10</t>
+          <t>2025-03</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Brunettin, Marilie</t>
+          <t>Brunettin, Mari; Marco Brunettin; Marco Brunettin, LL</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/Zoll payment.eml</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/46583 - Rechnung 250253_2025 vom 14.03.2025, Aufträge 31_25, 33_24, 34_24, 34_25, Mandant 42303.pdf</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -1552,22 +1552,22 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2024-02</t>
+          <t>2025-03</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Brunettin, Mari; Marco Brunettin; Marco Brunettin, LL</t>
+          <t>Arbeitsunfähigkeit, Entgeltbescheinigung bei; Brunettin, Mari; Marco Brunettin; Marco Brunettin, LL</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/Accountings 02-2024.eml::41261 - Rechnung 240303_2024 vom 27.03.2024, Aufträge 31_24, 33_24, 34_24, Mandant 42303.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/46851 - Rechnung 250303_2025 vom 31.03.2025, Aufträge 31_25, 33_25, 34_25, Mandant 42303.pdf</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -1579,76 +1579,76 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2025-02</t>
+          <t>2024-09</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>4</t>
+          <t/>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Arbeitsunfähigkeit, Entgeltbescheinigung bei; Brunettin, Mari; Marco Brunettin; Marco Brunettin, LL</t>
+          <t/>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/Accountings 02-2025.eml::46851 - Rechnung 250303_2025 vom 31.03.2025, Aufträge 31_25, 33_25, 34_25, Mandant 42303.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/CarlundCarla_RG424005125.pdf</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>LOW</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2024-03</t>
+          <t>2024-09</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>3</t>
+          <t/>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Brunettin, Mari; Marco Brunettin; Marco Brunettin, LL</t>
+          <t/>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/Accountings 03-2024.eml::41683 - Rechnung 240393_2024 vom 30.04.2024, Aufträge 31_24, 32_24, 33_24, 34_24, 98_24, Mandant 42303.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/CarlundCarla_RG424005157.pdf</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>LOW</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2024-04</t>
+          <t>2024-09</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Brunettin, Mari; Marco Brunettin; Marco Brunettin, LL</t>
+          <t>Brunettin, Marilie</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/Accountings 04-2024.eml::42108 - Rechnung 240498_2024 vom 30.05.2024, Aufträge 21_24, 31_24, 32_24, 33_24, 34_24, Mandant 42303.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Ihre Lohnauswertungen.eml</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -1660,22 +1660,22 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2024-06</t>
+          <t>2036-08</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Brunettin, Mari; EURPQ, Matodiev wage statement; Marco Brunettin; Marco Brunettin, LL; Stefanova, Yordanov</t>
+          <t>Logistikbetrieb Weißflog, Hohensteiner Str</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/Accountings 06-2024.eml::43029 - Rechnung 240697_2024 vom 31.07.2024, Aufträge 21_23, 21_24, 31_22, 31_23, 31_24, 33_24, 34_24, Mandant 42303.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Martin Zahariev Transporte 2036 08.01.2025 Scannermiete.pdf</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -1687,22 +1687,22 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2024-07</t>
+          <t>2054-07</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Brunettin, Mari; Marco Brunettin; Marco Brunettin, LL</t>
+          <t>Logistikbetrieb Weißflog, Hohensteiner Str</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/Accountings 07-2024.eml::43617 - Rechnung 240857_2024 vom 30.08.2024, Aufträge 31_24, 32_24, 33_24, 34_24, Mandant 42303.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Martin Zahariev Transporte 2054 07.02.2025 Scannermiete.pdf</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -1714,22 +1714,22 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2024-09</t>
+          <t>2058-08</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Brunettin, Mari; Marco Brunettin; Marco Brunettin, LL</t>
+          <t>Logistikbetrieb Weißflog, Hohensteiner Str</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/Accountings 09-2024.eml::44458 - Rechnung 241068_2024 vom 30.10.2024, Aufträge 31_24, 33_24, 34_24, Mandant 42303.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Martin Zahariev Transporte 2058 08.03.2025 Scannermiete.pdf</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -1741,103 +1741,103 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2024-10</t>
+          <t>2025-04</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>3</t>
+          <t/>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Brunettin, Mari; Marco Brunettin; Marco Brunettin, LL</t>
+          <t/>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/Accountings 10-2024.eml::45027 - Rechnung 241185_2024 vom 29.11.2024, Aufträge 31_24, 33_24, 34_24, Mandant 42303.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Rechnung 2765 Zahariev Hermes Scannermiete.pdf</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>LOW</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2024-11</t>
+          <t>2025-05</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>3</t>
+          <t/>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Brunettin, Mari; Marco Brunettin; Marco Brunettin, LL</t>
+          <t/>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/Accountings 11-2024.eml::45474 - Rechnung 241289_2024 vom 27.12.2024, Aufträge 21_24, 31_24, 32_24, 33_24, 34_24, 35_21, 35_24, 50_24, 98_24, Mandant 42303.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Rechnung 2777 Zahariev Hermes Unterstützungstouren.pdf</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>LOW</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2024-12</t>
+          <t>2025-05</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>3</t>
+          <t/>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Brunettin, Mari; Marco Brunettin; Marco Brunettin, LL</t>
+          <t/>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/Accountings 12-2024.eml::46583 - Rechnung 250253_2025 vom 14.03.2025, Aufträge 31_25, 33_24, 34_24, 34_25, Mandant 42303.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Rechnung 2778 Zahariev Hermes Scannermiete.pdf</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>LOW</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2024-01</t>
+          <t>2025-05</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Brunettin, Mari; Marco Brunettin; Marco Brunettin, LL</t>
+          <t>Bearbeitungsgebühr, Prüfung und Erstellung</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/accountings012024.zip::40850 - Rechnung 240213_2024 vom 29.01.2024, Aufträge 31_24, 32_23, 33_23, 33_24, 34_24, 98_24, Mandant 42303.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Rechnung 2782 Zahariev Hermes Bearbeitungsgebühr.pdf</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -1849,115 +1849,115 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2024-02</t>
+          <t>2025-06</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2</t>
+          <t/>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Marco Brunettin; Marco Brunettin, LL</t>
+          <t/>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/accountings012024.zip::40579 - Rechnung 240155_2024 vom 17.02.2024, Aufträge 31_23, 33_23, 34_23, Mandant 42303.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Rechnung 2788 Zahariev Hermes Scannermiete.pdf</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>LOW</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2023-12</t>
+          <t>2025-06</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2</t>
+          <t/>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Marco Brunettin; Marco Brunettin, LL</t>
+          <t/>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/accountings112023.zip::39739 - Rechnung 231128_2023 vom 28.12.2023, Aufträge 31_23, 32_23, 33_23, 34_23, 50_23, 98_23, Mandant 42303.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Rechnung 2789 Zahariev TF Touren.pdf</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>LOW</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2023-10</t>
+          <t>2025-06</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2</t>
+          <t/>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Marco Brunettin; Marco Brunettin, LL</t>
+          <t/>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/accountings112023.zip::90f3df27-1ca1-4b3a-9f1b-e33ffd37f10a.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Rechnung 2794 Zahariev KFZ Miete.pdf</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>LOW</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t/>
+          <t>2025-06</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t/>
+          <t>1</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t/>
+          <t>Bearbeitungsgebühr, Prüfung und Erstellung</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/awbonuses042024.zip::38389 - Vorgangsmappe Lohn - Auszahlungen Inflationsprämie.xlsx</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Rechnung 2799 Bearbeitungsgebühr 10.06.2025 Zahariev.pdf</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t/>
+          <t>2025-07</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -1972,7 +1972,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/awbonusfoodbonus032024.zip::38389 - Vorgangsmappe Lohn - Auszahlungen Inflationsprämie.xlsx</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Rechnung 2810 Zahariev TF Touren.pdf</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -1984,7 +1984,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2023-01</t>
+          <t>2025-07</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -1999,7 +1999,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/awbonusfoodbonus032024.zip::38389 - Vorgangsmappe Lohn - Working Hours 03-2024 .xlsx</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Rechnung 2811 Zahariev scannermiete.pdf</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -2011,61 +2011,61 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2025-05</t>
+          <t>2025-07</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t/>
+          <t>1</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t/>
+          <t>Bearbeitungsgebühr, Prüfung und Erstellung</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/fwdabrechnungmai2025.zip::gutschrift 66 Mai 2025 zahariev.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Rechnung 2813 zahariev bearbeitungsgebühr.pdf</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2024-09</t>
+          <t>2025-07</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>1</t>
+          <t/>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Logistikbetrieb Weißflog, Hohensteiner Str</t>
+          <t/>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/fwdabrechnungseptember.zip::Gutschrift 31-2024 Zahariev Martin 30.09.2024.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Rechnung 2814 zahariev bekleidung.pdf</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>LOW</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2025-04</t>
+          <t>2023-10</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2075,12 +2075,12 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Steuerbereinigter Schadenersatz, Schadenbetrag ohne Mehrwertsteuer</t>
+          <t>Dennis Kollmann, Marco Schlüter</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/fwdfwgutschriftrechnungen.zip::gutschrift 05.04. 2025 zahariev.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Unternehmerabrechnung - VP 120-2300157425.pdf</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -2092,7 +2092,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2025-03</t>
+          <t>2023-10</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2102,12 +2102,12 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Steuerbereinigter Schadenersatz, Schadenbetrag ohne Mehrwertsteuer</t>
+          <t>Dennis Kollmann, Marco Schlüter</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/fwdfwgutschriftrechnungen.zip::Rechnung 2766 Zahariev Hermes Sendungsverlust.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Unternehmerabrechnung - VP 120-2300157934.pdf</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -2119,61 +2119,61 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2025-04</t>
+          <t>2024-01</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t/>
+          <t>1</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t/>
+          <t>Dennis Kollmann, Marco Schlüter</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/fwdfwgutschriftrechnungen.zip::Rechnung 2764 Zahariev Hermes Kleidung.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Unternehmerabrechnung - VP 120-2400000826.pdf</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2025-04</t>
+          <t>2024-01</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t/>
+          <t>1</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t/>
+          <t>Dennis Kollmann, Marco Schlüter</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/fwdfwgutschriftrechnungen.zip::Rechnung 2765 Zahariev Hermes Scannermiete.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Unternehmerabrechnung - VP 120-2400000990.pdf</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2025-04</t>
+          <t>2024-01</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2183,12 +2183,12 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Bearbeitungsgebühr, Prüfung und Erstellung</t>
+          <t>Dennis Kollmann, Marco Schlüter</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/fwdfwgutschriftrechnungen.zip::Rechnung 2767 Zahariev Hermes Bearbeitungsgebuhr.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Unternehmerabrechnung - VP 120-2400001108-1.pdf</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -2200,88 +2200,88 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2025-06</t>
+          <t>2024-02</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t/>
+          <t>1</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t/>
+          <t>Dennis Kollmann, Marco Schlüter</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/fwdgsundrechnungen052025.zip::Rechnung 2788 Zahariev Hermes Scannermiete.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Unternehmerabrechnung - VP 120-2400017841.pdf</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2025-06</t>
+          <t>2024-02</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t/>
+          <t>1</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t/>
+          <t>Dennis Kollmann, Marco Schlüter</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/fwdgsundrechnungen052025.zip::Rechnung 2789 Zahariev TF Touren.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Unternehmerabrechnung - VP 120-2400018211.pdf</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2025-06</t>
+          <t>2024-01</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t/>
+          <t>1</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t/>
+          <t>Dennis Kollmann, Marco Schlüter</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/fwdgsundrechnungen052025.zip::Rechnung 2794 Zahariev KFZ Miete.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Unternehmerabrechnung - VP 120-2400035414.pdf</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2025-06</t>
+          <t>2024-01</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -2291,12 +2291,12 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Bearbeitungsgebühr, Prüfung und Erstellung</t>
+          <t>Dennis Kollmann, Marco Schlüter</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/fwdgsundrechnungen052025.zip::Rechnung 2799 Bearbeitungsgebühr 10.06.2025 Zahariev.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Unternehmerabrechnung - VP 120-2400035649.pdf</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -2308,7 +2308,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2024-11</t>
+          <t>2024-07</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2318,12 +2318,12 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Logistikbetrieb Weißflog, Hohensteiner Str</t>
+          <t>Logistikbetrieb Weißlog, Hohensteiner Str</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/fwdgutschriftundrechnungen.zip::Gutschrift 42-2024 Zahariev Martin 30.11.2024.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Docutain Dokument.pdf</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -2335,7 +2335,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2024-12</t>
+          <t>2025-04</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2350,7 +2350,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/fwdgutschriftundrechnungen.zip::Rechnung 2014 vom 05.12.2024 Sendungsverlust Zahariev.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/gutschrift 05.04. 2025 zahariev.pdf</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -2362,22 +2362,22 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2015-07</t>
+          <t>2024-07</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Bearbeitungsgebühr, Prüfung und Erstellung; Logistikbetrieb Weißflog, Hohensteiner Str</t>
+          <t>Logistikbetrieb Weißflog, Hohensteiner Str</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/fwdgutschriftundrechnungen.zip::Rechnung 2015 07.12.2024 Martin Zahariev.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Gutschrift 24-2024 Zahariev Martin 31.07.2024.pdf</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -2389,7 +2389,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2024-12</t>
+          <t>2024-09</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -2404,7 +2404,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/fwdgutschriftundrechnungen.zip::Rechnung 2023 vom 07.12.2024  Zahariev HERMES Bekleidung.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Gutschrift 31-2024 Zahariev Martin 30.09.2024.pdf</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -2416,22 +2416,22 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2024-01</t>
+          <t>2024-10</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Dennis Kollmann, Marco Schlüter</t>
+          <t>Goetz, Schneeberg; Logistikbetrieb Weißflog, Hohensteiner Str; Steuerbereinigter Schadenersatz, Schadenbetrag ohne Mehrwertsteuer</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/fwdihreabrechnungsunterlagen012024350690382950.zip::Unternehmerabrechnung - VP 120-2400035414.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Gutschrift 34-2024 Zahariev Martin 04.10.2024.pdf</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -2443,7 +2443,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2024-01</t>
+          <t>2024-10</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2453,12 +2453,12 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Dennis Kollmann, Marco Schlüter</t>
+          <t>Logistikbetrieb Weißflog, Hohensteiner Str</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/fwdihreabrechnungsunterlagen012024350690382950.zip::Unternehmerabrechnung - VP 120-2400035649.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Gutschrift 38-2024 Zahariev Martin 31.10.2024.pdf</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -2470,7 +2470,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2024-01</t>
+          <t>2024-11</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2480,12 +2480,12 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Dennis Kollmann, Marco Schlüter</t>
+          <t>Logistikbetrieb Weißflog, Hohensteiner Str</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/fwdihreabrechnungsunterlagen0120243506903829501.zip::Unternehmerabrechnung - VP 120-2400000826.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Gutschrift 42-2024 Zahariev Martin 30.11.2024.pdf</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
@@ -2497,7 +2497,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2024-01</t>
+          <t>2024-12</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2507,12 +2507,12 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Dennis Kollmann, Marco Schlüter</t>
+          <t>Logistikbetrieb Weißflog, Hohensteiner Str</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/fwdihreabrechnungsunterlagen0120243506903829501.zip::Unternehmerabrechnung - VP 120-2400000990.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Gutschrift 44-2024 Zahariev Martin 31.12.2024.pdf</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -2524,34 +2524,34 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2024-10</t>
+          <t>2025-05</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>1</t>
+          <t/>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Logistikbetrieb Weißflog, Hohensteiner Str</t>
+          <t/>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/fwdperemailsendengutschrift382024zaharievmartin3.zip::Gutschrift 38-2024 Zahariev Martin 31.10.2024.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/gutschrift 66 Mai 2025 zahariev.pdf</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>LOW</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2024-12</t>
+          <t>2025-06</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2561,12 +2561,12 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Logistikbetrieb Weißflog, Hohensteiner Str</t>
+          <t>Steuerbereinigter Schadenersatz, Schadenbetrag ohne Mehrwertsteuer</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/fwdperemailsendengutschrift442024zaharievmartin3.zip::Gutschrift 44-2024 Zahariev Martin 31.12.2024.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/gutschrift 71 2025 zahariev Sendungsverlust.pdf</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -2593,7 +2593,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/fwdperemailsendengutschriftapril2025zahariev_pdf.zip::gutschrift April 2025 zahariev.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/gutschrift April 2025 zahariev.pdf</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
@@ -2620,7 +2620,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/fwdperemailsendengutschriftmrz2025zahariev_pdf.zip::gutschrift märz 2025 zahariev.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/gutschrift märz 2025 zahariev.pdf</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -2632,34 +2632,34 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2025-02</t>
+          <t>2025-06</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>1</t>
+          <t/>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Logistikbetrieb Weißflog, Hohensteiner Str</t>
+          <t/>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/fwdperemailsendenleistungsnachweismartinzaharievfe.zip::Martin Zahariev Gutschrift 52 28.02.2025.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Gutschrift Zahariev 74 30.06.2025.pdf</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>LOW</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2024-07</t>
+          <t>2025-01</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2674,7 +2674,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/fwdperemailsendenleistungsnachweiszaharievjuli2024.zip::Gutschrift 24-2024 Zahariev Martin 31.07.2024.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Gutschrift 48 31.01.2025.pdf</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -2686,34 +2686,34 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2025-06</t>
+          <t>2025-02</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t/>
+          <t>2</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t/>
+          <t>Logistikbetrieb Weißflog, Hohensteiner Str; Steuerbereinigter Schadenersatz, Schadenbetrag ohne Mehrwertsteuer</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/fwdperemailsendenleistungsnachweiszaharievjuni25s.zip::Gutschrift Zahariev 74 30.06.2025.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Gutschrift 51 17.02.2025.pdf</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2025-01</t>
+          <t>2025-02</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2728,7 +2728,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/fwdperemailsendenmartinzaharievgutschrift4831_01_.zip::Martin Zahariev Gutschrift 48 31.01.2025.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Gutschrift 52 28.02.2025.pdf</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -2740,22 +2740,22 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2036-08</t>
+          <t>2025-03</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Logistikbetrieb Weißflog, Hohensteiner Str</t>
+          <t>Logistikbetrieb Weißflog, Hohensteiner Str; Steuerbereinigter Schadenersatz, Schadenbetrag ohne Mehrwertsteuer</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/fwdperemailsendenmartinzaharievtransporte203608_0.zip::Martin Zahariev Transporte 2036 08.01.2025 Scannermiete.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Gutschrift 55 08.03.2025.pdf</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
@@ -2767,7 +2767,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2037-08</t>
+          <t>2035-08</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -2777,12 +2777,12 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Steuerbereinigter Schadenersatz, Schadenbetrag ohne Mehrwertsteuer</t>
+          <t>Logistikbetrieb Weißflog, Hohensteiner Str</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/fwdperemailsendenmartinzaharievtransporte203608_0.zip::Martin Zahariev Transporte 2037 08.01.2025 Sendungsverluste.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Transporte 2035 08.01.2025 Hermes Bekleidung.pdf</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -2794,22 +2794,22 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2038-08</t>
+          <t>2037-08</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Bearbeitungsgebühr, Prüfung und Erstellung; Logistikbetrieb Weißflog, Hohensteiner Str</t>
+          <t>Steuerbereinigter Schadenersatz, Schadenbetrag ohne Mehrwertsteuer</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/fwdperemailsendenmartinzaharievtransporte203608_0.zip::Martin Zahariev Transporte 2038 08.01.2025 Bearbeitungsgebühr.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Transporte 2037 08.01.2025 Sendungsverluste.pdf</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
@@ -2821,22 +2821,22 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2035-08</t>
+          <t>2038-08</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Logistikbetrieb Weißflog, Hohensteiner Str</t>
+          <t>Bearbeitungsgebühr, Prüfung und Erstellung; Logistikbetrieb Weißflog, Hohensteiner Str</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/fwdperemailsendenmartinzaharievtransporte203608_0.zip::Martin Zahariev Transporte 2035 08.01.2025 Hermes Bekleidung.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Transporte 2038 08.01.2025 Bearbeitungsgebühr.pdf</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -2848,7 +2848,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2054-07</t>
+          <t>2055-07</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -2858,12 +2858,12 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Logistikbetrieb Weißflog, Hohensteiner Str</t>
+          <t>Steuerbereinigter Schadenersatz, Schadenbetrag ohne Mehrwertsteuer</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/fwdperemailsendenmartinzaharievtransporte205407_0.zip::Martin Zahariev Transporte 2054 07.02.2025 Scannermiete.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Transporte 2055 07.02.2025 Sendungsverluste.pdf</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -2875,22 +2875,22 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2055-07</t>
+          <t>2056-07</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Steuerbereinigter Schadenersatz, Schadenbetrag ohne Mehrwertsteuer</t>
+          <t>Bearbeitungsgebühr, Prüfung und Erstellung; Logistikbetrieb Weißflog, Hohensteiner Str</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/fwdperemailsendenmartinzaharievtransporte205407_0.zip::Martin Zahariev Transporte 2055 07.02.2025 Sendungsverluste.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Transporte 2056 07.02.2025 Bearbeitungsgebühr.pdf</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -2902,22 +2902,22 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2056-07</t>
+          <t>2057-07</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Bearbeitungsgebühr, Prüfung und Erstellung; Logistikbetrieb Weißflog, Hohensteiner Str</t>
+          <t>Logistikbetrieb Weißflog, Hohensteiner Str</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/fwdperemailsendenmartinzaharievtransporte205407_0.zip::Martin Zahariev Transporte 2056 07.02.2025 Bearbeitungsgebühr.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Transporte 2057 07.02.2025 Hermes Bekleidung.pdf</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -2929,22 +2929,22 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2057-07</t>
+          <t>2069-08</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Logistikbetrieb Weißflog, Hohensteiner Str</t>
+          <t>Logistikbetrieb Weißflog, Hohensteiner Str; Steuerbereinigter Schadenersatz, Schadenbetrag ohne Mehrwertsteuer</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/fwdperemailsendenmartinzaharievtransporte205407_0.zip::Martin Zahariev Transporte 2057 07.02.2025 Hermes Bekleidung.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Transporte 2069 08.03.2025 Sendungsverluste.pdf</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -2971,7 +2971,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/fwdperemailsendenmartinzaharievtransporte207008_0.zip::Martin Zahariev Transporte 2070 08.03.2025 Sendungsverluste.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Transporte 2070 08.03.2025 Sendungsverluste.pdf</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -2983,22 +2983,22 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2069-08</t>
+          <t>2024-12</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Logistikbetrieb Weißflog, Hohensteiner Str; Steuerbereinigter Schadenersatz, Schadenbetrag ohne Mehrwertsteuer</t>
+          <t>Steuerbereinigter Schadenersatz, Schadenbetrag ohne Mehrwertsteuer</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/fwdperemailsendenmartinzaharievtransporte207008_0.zip::Martin Zahariev Transporte 2069 08.03.2025 Sendungsverluste.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Rechnung 2014 vom 05.12.2024 Sendungsverlust Zahariev.pdf</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -3010,115 +3010,115 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2025-05</t>
+          <t>2015-07</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t/>
+          <t>2</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t/>
+          <t>Bearbeitungsgebühr, Prüfung und Erstellung; Logistikbetrieb Weißflog, Hohensteiner Str</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/fwdperemailsendenrechnung2778zaharievhermesscanne.zip::Rechnung 2778 Zahariev Hermes Scannermiete.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Rechnung 2015 07.12.2024 Martin Zahariev.pdf</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2025-05</t>
+          <t>2024-12</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t/>
+          <t>1</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t/>
+          <t>Logistikbetrieb Weißflog, Hohensteiner Str</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/fwdperemailsendenrechnung2778zaharievhermesscanne.zip::Rechnung 2777 Zahariev Hermes Unterstützungstouren.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Rechnung 2023 vom 07.12.2024  Zahariev HERMES Bekleidung.pdf</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2025-05</t>
+          <t>2025-04</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>1</t>
+          <t/>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Bearbeitungsgebühr, Prüfung und Erstellung</t>
+          <t/>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/fwdperemailsendenrechnung2778zaharievhermesscanne.zip::Rechnung 2782 Zahariev Hermes Bearbeitungsgebühr.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Rechnung 2764 Zahariev Hermes Kleidung.pdf</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>LOW</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2025-07</t>
+          <t>2025-03</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t/>
+          <t>1</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t/>
+          <t>Steuerbereinigter Schadenersatz, Schadenbetrag ohne Mehrwertsteuer</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/fwdrechnungenaus062025.zip::Rechnung 2814 zahariev bekleidung.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Rechnung 2766 Zahariev Hermes Sendungsverlust.pdf</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2025-07</t>
+          <t>2025-04</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -3133,7 +3133,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/fwdrechnungenaus062025.zip::Rechnung 2813 zahariev bearbeitungsgebühr.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Rechnung 2767 Zahariev Hermes Bearbeitungsgebuhr.pdf</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
@@ -3145,295 +3145,52 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2025-07</t>
+          <t>2024-08</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t/>
+          <t>3</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t/>
+          <t>Chemnitz , Sachs; Motoren-Frech, Uwe; Thomas Frech GbR, Hohensteiner Straße</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/fwdrechnungenaus062025.zip::Rechnung 2811 Zahariev scannermiete.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/11_Contribution_Lists/RE-53380_2024 13.08.2024 09_17_16.pdf</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2025-07</t>
+          <t>2024-09</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t/>
+          <t>3</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t/>
+          <t>Chemnitz , Sachs; Motoren-Frech, Uwe; Thomas Frech GbR, Hohensteiner Straße</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/fwdrechnungenaus062025.zip::Rechnung 2810 Zahariev TF Touren.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/11_Contribution_Lists/RE-53652_2024 20.09.2024 10_56_50.pdf</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="B119" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="C119" t="inlineStr">
-        <is>
-          <t>Boulevard Royal, L; Der Verkäufer behält sich vor, Verarbeitungsaufträge abzulehnen; E-Mail, Fax oder Brief; EE Amsterdam, Niederlande; Grafiken in den vom Verkäufer vorgegebenen Dateiformaten, Formatierungen; Kennedy, L; Reklamationen, Widerrufserklärungen und; Reklamationen, Widerrufserklärungen und -zusendungen oder Gutschriften; Stockholm, Schweden; Urheber-, Marken- und Persönlichkeitsrechte; Versendung, Retouren; Ware, Lieferzeit; Zahlungsabwicklung über die TeamBank AG Nürnberg, Beuthener Straße; Überweisungsgebühren, Wechselkursgebühren</t>
-        </is>
-      </c>
-      <c r="D119" t="inlineStr">
-        <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/ihrebestellung465795beiwebergmbh.zip::agb_doc.pdf</t>
-        </is>
-      </c>
-      <c r="E119" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="B120" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="C120" t="inlineStr">
-        <is>
-          <t>Herleshausen, Deutschland; Post versandter Brief, Telefax oder E-Mail; Weber GmbH, Sülzbach</t>
-        </is>
-      </c>
-      <c r="D120" t="inlineStr">
-        <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/ihrebestellung465795beiwebergmbh.zip::widerruf_doc.pdf</t>
-        </is>
-      </c>
-      <c r="E120" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" t="inlineStr">
-        <is>
-          <t>2025-06</t>
-        </is>
-      </c>
-      <c r="B121" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="C121" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D121" t="inlineStr">
-        <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/ihrelohnauswertungen.zip::working hours 06.2025  _____.xlsx</t>
-        </is>
-      </c>
-      <c r="E121" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" t="inlineStr">
-        <is>
-          <t>2018-05</t>
-        </is>
-      </c>
-      <c r="B122" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="C122" t="inlineStr">
-        <is>
-          <t>BIG direkt gesund, Rheinische Straße; Dortmund, Deutschland; Peter Kaetsch, Markus Bäumer</t>
-        </is>
-      </c>
-      <c r="D122" t="inlineStr">
-        <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/ihrelohnauswertungen3333.zip::BIG_Arbeitgeber_SEPA_Lastschriftmandat.pdf</t>
-        </is>
-      </c>
-      <c r="E122" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" t="inlineStr">
-        <is>
-          <t>2025-04</t>
-        </is>
-      </c>
-      <c r="B123" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="C123" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D123" t="inlineStr">
-        <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/ihrelohnauswertungenapril2025.zip::working hours 04.2025.xlsx</t>
-        </is>
-      </c>
-      <c r="E123" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" t="inlineStr">
-        <is>
-          <t>2023-01</t>
-        </is>
-      </c>
-      <c r="B124" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="C124" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D124" t="inlineStr">
-        <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/ihrelohnauswertungendezember2024.zip::working hours 12.2024.xlsx</t>
-        </is>
-      </c>
-      <c r="E124" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="B125" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="C125" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D125" t="inlineStr">
-        <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/testpayslip.zip::38389 - Vorgangsmappe Lohn - 38389 - Aktualisiert- Auszahlungen Inflationsprämie.xlsx</t>
-        </is>
-      </c>
-      <c r="E125" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="B126" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="C126" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D126" t="inlineStr">
-        <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/updatedworkinghoursinflationsprmie.zip::38389 - Vorgangsmappe Lohn - Auszahlungen Inflationsprämie.xlsx</t>
-        </is>
-      </c>
-      <c r="E126" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" t="inlineStr">
-        <is>
-          <t>2024-01</t>
-        </is>
-      </c>
-      <c r="B127" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="C127" t="inlineStr">
-        <is>
-          <t>Akkreditiert durch DAkkS, Registriernummer; Berlin-Charlottenburg, HRB; Präqualifikation Kurier-, Express- und Paketdienstleistern i; ZERTIFIZIERUNG BAU GMBH, Kronenstraße</t>
-        </is>
-      </c>
-      <c r="D127" t="inlineStr">
-        <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting/wgprqualifikationkepkdnr_60222rechnungjahresgeb.zip::20240123_60222_10160_Rechnung.pdf</t>
-        </is>
-      </c>
-      <c r="E127" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>

</xml_diff>